<commit_message>
Fix the date freeze, add sub-events to event types for the event name
- A year half typed in (0202 on the way to 2026) sent the festival code into an endless
  loop. Dates now always keep a four-digit year, the festival code skips years that are not
  real, and such a year is refused on save.
- Sub-events per event type (0023): Wedding has Haldi, Mehndi, Sangeet, Garba, Mandap
  Muhurat, Wedding Day and Reception. Set in Settings, Event types, or by the import's new
  Sub events column, which adds new ones to a type already there.
- The service's Event Name is a searchable drop-down of those sub-events that also takes a
  typed name. The food service no longer fills it; a blank one is saved as Service N.
- The service card puts the 12-hour time pickers two to a row so they no longer overlap.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import-examples/09 Event types.xlsx
+++ b/docs/import-examples/09 Event types.xlsx
@@ -23,29 +23,54 @@
         </r>
       </text>
     </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t>Optional. The events inside it, separated by ; e.g. Haldi; Sangeet; Reception. They are suggested as the Event Name of each catering service. For a type you already have, new ones are added to its list.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Event type</t>
   </si>
   <si>
+    <t>Sub events</t>
+  </si>
+  <si>
     <t>Wedding</t>
   </si>
   <si>
+    <t>Haldi; Mehndi; Sangeet; Garba; Mandap Muhurat; Wedding Day; Reception</t>
+  </si>
+  <si>
     <t>Engagement</t>
   </si>
   <si>
+    <t>Ring Ceremony; Engagement Lunch; Engagement Dinner</t>
+  </si>
+  <si>
     <t>Birthday Party</t>
   </si>
   <si>
+    <t>Cake Cutting; Birthday Party; Birthday Lunch</t>
+  </si>
+  <si>
     <t>Griha Shanti</t>
   </si>
   <si>
+    <t>Griha Shanti Puja; Griha Shanti Lunch</t>
+  </si>
+  <si>
     <t>Corporate Lunch</t>
+  </si>
+  <si>
+    <t>Conference Lunch; Team Lunch</t>
   </si>
 </sst>
 </file>
@@ -65,7 +90,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,6 +100,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB4372B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6B6158"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,9 +120,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -434,40 +467,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>